<commit_message>
Update docs: dashboard data, assets and reports
Regenerate and update documentation assets: add docs/.nojekyll, rename S Curve file to a simplified name and remove obsolete S Curve binary, update S_Curve_Dashboard_Source.xlsx and fully regenerate docs/data/dashboard-data.json with new metrics/timestamps, update docs/index.html and static CSS/JS (styles.css, app.js). Replace/remove several report files and add two new PDF report options (WTE_CEO_Premium_Report_Option_A/B.pdf) and update WTE_Dashboard_Report.xlsx.
</commit_message>
<xml_diff>
--- a/docs/reports/WTE_Dashboard_Report.xlsx
+++ b/docs/reports/WTE_Dashboard_Report.xlsx
@@ -828,7 +828,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generato: 2026-05-20 11:03</t>
+          <t>Generato: 2026-05-22 12:52</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1459,7 +1459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G122"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>8.5.2.2</t>
+          <t>8.5.1</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Office kitchen furniture  ECd_36</t>
+          <t>Internet Connection ECd_37</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -1530,10 +1530,10 @@
         </is>
       </c>
       <c r="E2" s="13" t="n">
-        <v>46070</v>
+        <v>46073</v>
       </c>
       <c r="F2" s="6" t="n">
-        <v>13414.64</v>
+        <v>27350</v>
       </c>
       <c r="G2" s="5" t="n"/>
     </row>
@@ -1545,12 +1545,12 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>8.5.1</t>
+          <t>8.1.3.3</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Internet Connection ECd_37</t>
+          <t>Open order - sanitary industry assortment ECd_39</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -1559,10 +1559,10 @@
         </is>
       </c>
       <c r="E3" s="13" t="n">
-        <v>46073</v>
+        <v>46077</v>
       </c>
       <c r="F3" s="6" t="n">
-        <v>27350</v>
+        <v>30000</v>
       </c>
       <c r="G3" s="5" t="n"/>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>8.1.3.3</t>
+          <t>8.1.3.4</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Open order - sanitary industry assortment ECd_39</t>
+          <t>Open order - sanitary industry assortment ECd_40</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -1603,12 +1603,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>8.1.3.4</t>
+          <t>1.2.2</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Open order - sanitary industry assortment ECd_40</t>
+          <t>Detailed design: boiler support steel structure and equipment support structures</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -1617,10 +1617,10 @@
         </is>
       </c>
       <c r="E5" s="13" t="n">
-        <v>46077</v>
+        <v>46080</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>30000</v>
+        <v>943000</v>
       </c>
       <c r="G5" s="5" t="n"/>
     </row>
@@ -1632,12 +1632,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>8.4.1.1</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Detailed design: boiler support steel structure and equipment support structures</t>
+          <t>Personal Occupational Health and Safety Equipment ECd_43</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -1646,10 +1646,10 @@
         </is>
       </c>
       <c r="E6" s="13" t="n">
-        <v>46080</v>
+        <v>46090</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>943000</v>
+        <v>30000</v>
       </c>
       <c r="G6" s="5" t="n"/>
     </row>
@@ -1661,12 +1661,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>8.4.1.1</t>
+          <t>8.3.1.2</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Personal Occupational Health and Safety Equipment ECd_43</t>
+          <t>Generator rental ECd_44</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -1675,10 +1675,10 @@
         </is>
       </c>
       <c r="E7" s="13" t="n">
-        <v>46090</v>
+        <v>46096</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>30000</v>
+        <v>23904</v>
       </c>
       <c r="G7" s="5" t="n"/>
     </row>
@@ -1690,12 +1690,12 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>8.3.1.2</t>
+          <t>8.7.1.6</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Generator rental ECd_44</t>
+          <t>Purchase of road signs ECd_42</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1707,7 +1707,7 @@
         <v>46096</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>23904</v>
+        <v>2000</v>
       </c>
       <c r="G8" s="5" t="n"/>
     </row>
@@ -1719,12 +1719,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>8.7.1.6</t>
+          <t>8.7.1.7</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Purchase of road signs ECd_42</t>
+          <t>Purchase of rubble for the construction of storage yards and work platforms ECd_45</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -1736,7 +1736,7 @@
         <v>46096</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>2000</v>
+        <v>83200</v>
       </c>
       <c r="G9" s="5" t="n"/>
     </row>
@@ -1748,12 +1748,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>8.7.1.7</t>
+          <t>2.11.5.3</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Purchase of rubble for the construction of storage yards and work platforms ECd_45</t>
+          <t>Concrete slab installation on the ground</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1762,12 +1762,16 @@
         </is>
       </c>
       <c r="E10" s="13" t="n">
-        <v>46096</v>
+        <v>46106</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>83200</v>
-      </c>
-      <c r="G10" s="5" t="n"/>
+        <v>1735392.78</v>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Agnieszka Zając</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -1777,12 +1781,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2.11.5.3</t>
+          <t>2.14.2.2</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Concrete slab installation on the ground</t>
+          <t>External road - aggregate delivery ECd_46</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1794,7 +1798,7 @@
         <v>46106</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>1735392.78</v>
+        <v>134400</v>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
@@ -1810,12 +1814,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>2.14.2.2</t>
+          <t>2.4.1</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>External road - aggregate delivery ECd_46</t>
+          <t>Insulation - work</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1827,7 +1831,7 @@
         <v>46106</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>134400</v>
+        <v>733045.25</v>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
@@ -1843,12 +1847,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2.4.1</t>
+          <t>2.5.1.3</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Insulation - work</t>
+          <t>Construction of reinforced concrete foundations and underground structures</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1860,7 +1864,7 @@
         <v>46106</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>733045.25</v>
+        <v>5276959.37</v>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
@@ -1876,12 +1880,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>2.5.1.3</t>
+          <t>2.5.2.1</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Construction of reinforced concrete foundations and underground structures</t>
+          <t>Reinforced concrete structure of the above-ground part of the B1 building - delivery and assembly of prefabricated elements</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1893,11 +1897,11 @@
         <v>46106</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>5276959.37</v>
+        <v>16616880</v>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Agnieszka Zając</t>
+          <t>Jan Szczubiał</t>
         </is>
       </c>
     </row>
@@ -1909,12 +1913,12 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2.5.2.1</t>
+          <t>2.5.2.2.3</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Reinforced concrete structure of the above-ground part of the B1 building - delivery and assembly of prefabricated elements</t>
+          <t>Reinforced concrete structure of the above-ground part of the B3 building - delivery and assembly of prefabricated elements</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1926,7 +1930,7 @@
         <v>46106</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>16616880</v>
+        <v>2115950</v>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
@@ -1942,12 +1946,12 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>2.5.2.2.3</t>
+          <t>2.5.2.2.4</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Reinforced concrete structure of the above-ground part of the B3 building - delivery and assembly of prefabricated elements</t>
+          <t>Reinforced concrete structure of the above-ground part of the other buildings</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1959,7 +1963,7 @@
         <v>46106</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>2115950</v>
+        <v>708072.75</v>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
@@ -1975,12 +1979,12 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2.5.2.2.4</t>
+          <t>2.6.2.1</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Reinforced concrete structure of the above-ground part of the other buildings</t>
+          <t>Precast reinforced concrete structure of facility B3 (change from steel structure compared to the acquisition stage)</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -1992,11 +1996,11 @@
         <v>46106</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>708072.75</v>
+        <v>1004390</v>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Jan Szczubiał</t>
+          <t>Robert Klimczak</t>
         </is>
       </c>
     </row>
@@ -2008,12 +2012,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>2.6.2.1</t>
+          <t>2.6.3.1</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Precast reinforced concrete structure of facility B3 (change from steel structure compared to the acquisition stage)</t>
+          <t>Precast reinforced concrete structure of facility B4 (change from steel structure compared to the acquisition stage)</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -2025,7 +2029,7 @@
         <v>46106</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>1004390</v>
+        <v>246780</v>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
@@ -2041,12 +2045,12 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2.6.3.1</t>
+          <t>2.14.2.1</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Precast reinforced concrete structure of facility B4 (change from steel structure compared to the acquisition stage)</t>
+          <t>External road- sub-base construction</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -2055,14 +2059,14 @@
         </is>
       </c>
       <c r="E19" s="13" t="n">
-        <v>46106</v>
+        <v>46122</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>246780</v>
+        <v>250640</v>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Robert Klimczak</t>
+          <t>Agnieszka Zając</t>
         </is>
       </c>
     </row>
@@ -2074,12 +2078,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>2.14.2.1</t>
+          <t>8.3.1.1</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>External road- sub-base construction</t>
+          <t>Electricity Costs</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -2091,13 +2095,9 @@
         <v>46122</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>250640</v>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>Agnieszka Zając</t>
-        </is>
-      </c>
+        <v>100000</v>
+      </c>
+      <c r="G20" s="5" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -2107,12 +2107,12 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>8.3.1.1</t>
+          <t>8.7.1.4</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Electricity Costs</t>
+          <t>Construction of aggregate squares</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -2124,9 +2124,13 @@
         <v>46122</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>100000</v>
-      </c>
-      <c r="G21" s="5" t="n"/>
+        <v>124700</v>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Agnieszka Zając</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -2136,12 +2140,12 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>8.7.1.4</t>
+          <t>8.8.4</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Construction of aggregate squares</t>
+          <t>Removing collisions related to site preparation and construction</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -2153,13 +2157,9 @@
         <v>46122</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>124700</v>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>Agnieszka Zając</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G22" s="5" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
@@ -2169,12 +2169,12 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>8.8.4</t>
+          <t>8.8.4.1</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Removing collisions related to site preparation and construction</t>
+          <t>Removal of existing reinforced concrete foundations in the vicinity of Building B2</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -2186,7 +2186,7 @@
         <v>46122</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="G23" s="5" t="n"/>
     </row>
@@ -2198,12 +2198,12 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>8.8.4.1</t>
+          <t>5.10.2</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Removal of existing reinforced concrete foundations in the vicinity of Building B2</t>
+          <t>Auxiliary crane and hoists for the maintenance of the steam turbine</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -2212,12 +2212,16 @@
         </is>
       </c>
       <c r="E24" s="13" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>50000</v>
-      </c>
-      <c r="G24" s="5" t="n"/>
+        <v>499000</v>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Magdalena Białorucka</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -2227,12 +2231,12 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>5.10.2</t>
+          <t>5.2.1</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Auxiliary crane and hoists for the maintenance of the steam turbine</t>
+          <t>Overhead crane, grab and operator seat + Spare Grab</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -2244,7 +2248,7 @@
         <v>46125</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>499000</v>
+        <v>8701000</v>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
@@ -2260,12 +2264,12 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>5.2.1</t>
+          <t>5.11</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Overhead crane, grab and operator seat + Spare Grab</t>
+          <t>Stack</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -2274,10 +2278,10 @@
         </is>
       </c>
       <c r="E26" s="13" t="n">
-        <v>46125</v>
+        <v>46127</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>8701000</v>
+        <v>1498200</v>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
@@ -2293,12 +2297,12 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>5.11</t>
+          <t>5.4.1.1</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Stack</t>
+          <t>Boiler - pressure parts</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -2310,11 +2314,11 @@
         <v>46127</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>1498200</v>
+        <v>45990000</v>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Magdalena Białorucka</t>
+          <t>Roger Gołombek</t>
         </is>
       </c>
     </row>
@@ -2326,12 +2330,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>5.4.1.1</t>
+          <t>8.3.5</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Boiler - pressure parts</t>
+          <t>Construction Waste Removal  ECd_38</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -2343,13 +2347,9 @@
         <v>46127</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>45990000</v>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>Roger Gołombek</t>
-        </is>
-      </c>
+        <v>290720</v>
+      </c>
+      <c r="G28" s="5" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -2359,12 +2359,12 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>8.3.5</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Construction Waste Removal  ECd_38</t>
+          <t>Drainage</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -2373,10 +2373,10 @@
         </is>
       </c>
       <c r="E29" s="13" t="n">
-        <v>46127</v>
+        <v>46129</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>290720</v>
+        <v>0</v>
       </c>
       <c r="G29" s="5" t="n"/>
     </row>
@@ -2388,12 +2388,12 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.3.1</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Rental of an drainage pump ECd_49</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -2405,7 +2405,7 @@
         <v>46129</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>0</v>
+        <v>4600</v>
       </c>
       <c r="G30" s="5" t="n"/>
     </row>
@@ -2417,12 +2417,12 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2.3.1</t>
+          <t>2.3.2</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Rental of an drainage pump ECd_49</t>
+          <t xml:space="preserve">Mobilization, installation and leasing of a wellpoint system including pumps ECd_50 </t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -2434,7 +2434,7 @@
         <v>46129</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>4600</v>
+        <v>70000</v>
       </c>
       <c r="G31" s="5" t="n"/>
     </row>
@@ -2446,12 +2446,12 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>2.3.2</t>
+          <t>1.2.4</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mobilization, installation and leasing of a wellpoint system including pumps ECd_50 </t>
+          <t xml:space="preserve">Electrical &amp; I/C detailed design </t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -2460,10 +2460,10 @@
         </is>
       </c>
       <c r="E32" s="13" t="n">
-        <v>46129</v>
+        <v>46134</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>70000</v>
+        <v>1620000</v>
       </c>
       <c r="G32" s="5" t="n"/>
     </row>
@@ -2475,12 +2475,12 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>1.2.4</t>
+          <t>3.1.1</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electrical &amp; I/C detailed design </t>
+          <t>Delivery and installation of electrical equipment</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -2492,9 +2492,13 @@
         <v>46134</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>1620000</v>
-      </c>
-      <c r="G33" s="5" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>Radosław Zdancewicz</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
@@ -2504,7 +2508,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>3.1.1</t>
+          <t>3.1.1.1</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -2521,7 +2525,7 @@
         <v>46134</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>0</v>
+        <v>27750000</v>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
@@ -2537,12 +2541,12 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>3.1.1.1</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Delivery and installation of electrical equipment</t>
+          <t>Teletechnical installations</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
@@ -2554,7 +2558,7 @@
         <v>46134</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>27750000</v>
+        <v>1750000</v>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
@@ -2570,12 +2574,12 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.4.1</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Teletechnical installations</t>
+          <t>Automation system and instrumentation, communication networks and control room devices</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -2587,7 +2591,7 @@
         <v>46134</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>1750000</v>
+        <v>0</v>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
@@ -2603,7 +2607,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>3.4.1</t>
+          <t>3.4.1.1</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -2620,7 +2624,7 @@
         <v>46134</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>0</v>
+        <v>6280000</v>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
@@ -2636,12 +2640,12 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>3.4.1.1</t>
+          <t>6.4.1</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Automation system and instrumentation, communication networks and control room devices</t>
+          <t>Extension of the guarantee and warranty period to 48 months for electrical, technical and I&amp;C works</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -2653,7 +2657,7 @@
         <v>46134</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>6280000</v>
+        <v>350000</v>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
@@ -2669,28 +2673,28 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>6.4.1</t>
+          <t>5.10.1</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Extension of the guarantee and warranty period to 48 months for electrical, technical and I&amp;C works</t>
+          <t>Steam turbine - gear box - generator. Including accessories: oil system, coolers, insulation, pipes and valves, control panel, protection panel, synchro system etc.</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>PCT/approval</t>
         </is>
       </c>
       <c r="E39" s="13" t="n">
-        <v>46134</v>
+        <v>46137</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>350000</v>
+        <v>0</v>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Radosław Zdancewicz</t>
+          <t>Magdalena Białorucka / Stanisław Rucki</t>
         </is>
       </c>
     </row>
@@ -2702,12 +2706,12 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>5.10.1</t>
+          <t>5.8.1</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Steam turbine - gear box - generator. Including accessories: oil system, coolers, insulation, pipes and valves, control panel, protection panel, synchro system etc.</t>
+          <t>Chain conveyor under grate + Bottom ash extractor + Vibrating table / bulk screen</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
@@ -2719,11 +2723,11 @@
         <v>46137</v>
       </c>
       <c r="F40" s="6" t="n">
-        <v>0</v>
+        <v>1462000</v>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Magdalena Białorucka / Stanisław Rucki</t>
+          <t>Stanisław Rucki</t>
         </is>
       </c>
     </row>
@@ -2735,30 +2739,26 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>5.8.1</t>
+          <t>2.4.2</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Chain conveyor under grate + Bottom ash extractor + Vibrating table / bulk screen</t>
+          <t>Insulation – supply – Hydrostop ECd_51</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>PCT/approval</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="E41" s="13" t="n">
-        <v>46137</v>
+        <v>46142</v>
       </c>
       <c r="F41" s="6" t="n">
-        <v>1462000</v>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>Stanisław Rucki</t>
-        </is>
-      </c>
+        <v>31352</v>
+      </c>
+      <c r="G41" s="5" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
@@ -2768,12 +2768,12 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>2.4.2</t>
+          <t>2.4.3</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Insulation – supply – Hydrostop ECd_51</t>
+          <t>Insulation – supply – foil, compound ECd_14</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
@@ -2785,7 +2785,7 @@
         <v>46142</v>
       </c>
       <c r="F42" s="6" t="n">
-        <v>31352</v>
+        <v>27600</v>
       </c>
       <c r="G42" s="5" t="n"/>
     </row>
@@ -2797,12 +2797,12 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>2.4.3</t>
+          <t>8.1.1.1</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Insulation – supply – foil, compound ECd_14</t>
+          <t>Purchase of temporary stairs ECd_48</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
@@ -2814,7 +2814,7 @@
         <v>46142</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>27600</v>
+        <v>17530</v>
       </c>
       <c r="G43" s="5" t="n"/>
     </row>
@@ -2826,12 +2826,12 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>8.1.1.1</t>
+          <t>8.1.1.2</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Purchase of temporary stairs ECd_48</t>
+          <t>Meals ECd_53</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
@@ -2843,7 +2843,7 @@
         <v>46142</v>
       </c>
       <c r="F44" s="6" t="n">
-        <v>17530</v>
+        <v>5711</v>
       </c>
       <c r="G44" s="5" t="n"/>
     </row>
@@ -2855,12 +2855,12 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>8.1.1.2</t>
+          <t>8.7.1.8</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Meals ECd_53</t>
+          <t>Installation of road markings and traffic signs ECd_52</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
@@ -2872,38 +2872,42 @@
         <v>46142</v>
       </c>
       <c r="F45" s="6" t="n">
-        <v>5711</v>
+        <v>920</v>
       </c>
       <c r="G45" s="5" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Closed last 3 months</t>
+          <t>Next orders 3 months</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>8.7.1.8</t>
+          <t>5.13.7</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Installation of road markings and traffic signs ECd_52</t>
+          <t>Demi water system including storage tank 100m3 and piping</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="E46" s="13" t="n">
-        <v>46142</v>
+        <v>46169</v>
       </c>
       <c r="F46" s="6" t="n">
-        <v>920</v>
-      </c>
-      <c r="G46" s="5" t="n"/>
+        <v>3010000</v>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>Magdalena Białorucka</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
@@ -2913,12 +2917,12 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>5.13.7</t>
+          <t>2.7</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Demi water system including storage tank 100m3 and piping</t>
+          <t>Brick walls</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
@@ -2927,16 +2931,12 @@
         </is>
       </c>
       <c r="E47" s="13" t="n">
-        <v>46169</v>
+        <v>46173</v>
       </c>
       <c r="F47" s="6" t="n">
-        <v>3010000</v>
-      </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>Magdalena Białorucka</t>
-        </is>
-      </c>
+        <v>687451.25</v>
+      </c>
+      <c r="G47" s="5" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
@@ -2946,12 +2946,12 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>2.7</t>
+          <t>5.2.2</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Brick walls</t>
+          <t>Trapdoors for grab maintenance</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
@@ -2963,7 +2963,7 @@
         <v>46173</v>
       </c>
       <c r="F48" s="6" t="n">
-        <v>687451.25</v>
+        <v>81600</v>
       </c>
       <c r="G48" s="5" t="n"/>
     </row>
@@ -2975,24 +2975,24 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>5.2.2</t>
+          <t>1.2.6.1</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Trapdoors for grab maintenance</t>
+          <t>Ducts design</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>enquiry</t>
         </is>
       </c>
       <c r="E49" s="13" t="n">
-        <v>46173</v>
+        <v>46174</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>81600</v>
+        <v>0</v>
       </c>
       <c r="G49" s="5" t="n"/>
     </row>
@@ -3004,24 +3004,24 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>1.2.6.1</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Ducts design</t>
+          <t xml:space="preserve">Explosion hazard assessment </t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>enquiry</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="E50" s="13" t="n">
         <v>46174</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="G50" s="5" t="n"/>
     </row>
@@ -3033,26 +3033,30 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>5.10.4</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Explosion hazard assessment </t>
+          <t>Feed water tank and Deaerator</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>negotiation</t>
         </is>
       </c>
       <c r="E51" s="13" t="n">
         <v>46174</v>
       </c>
       <c r="F51" s="6" t="n">
-        <v>120000</v>
-      </c>
-      <c r="G51" s="5" t="n"/>
+        <v>1000000</v>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>Magdalena Białorucka</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
@@ -3062,28 +3066,28 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>5.10.4</t>
+          <t>5.9</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Feed water tank and Deaerator</t>
+          <t>Bottom ash / slag valorization</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>negotiation</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="E52" s="13" t="n">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="F52" s="6" t="n">
-        <v>1000000</v>
+        <v>8271000</v>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>Magdalena Białorucka</t>
+          <t>Roger Gołombek</t>
         </is>
       </c>
     </row>
@@ -3095,12 +3099,12 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>5.9</t>
+          <t>5.8.2</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Bottom ash / slag valorization</t>
+          <t>Belt conveyors</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
@@ -3109,14 +3113,14 @@
         </is>
       </c>
       <c r="E53" s="13" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
       <c r="F53" s="6" t="n">
-        <v>8271000</v>
+        <v>2347800</v>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>Roger Gołombek</t>
+          <t>Stanisław Rucki</t>
         </is>
       </c>
     </row>
@@ -3128,28 +3132,28 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>5.8.2</t>
+          <t>5.10.3</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Belt conveyors</t>
+          <t>Air cooled condenser</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>enquiry</t>
         </is>
       </c>
       <c r="E54" s="13" t="n">
-        <v>46176</v>
+        <v>46178</v>
       </c>
       <c r="F54" s="6" t="n">
-        <v>2347800</v>
+        <v>9000000</v>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>Stanisław Rucki</t>
+          <t>Roger Gołombek</t>
         </is>
       </c>
     </row>
@@ -3161,12 +3165,12 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>5.10.3</t>
+          <t>2.5.2.3</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Air cooled condenser</t>
+          <t>Supply of reinforcing steel</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
@@ -3175,14 +3179,14 @@
         </is>
       </c>
       <c r="E55" s="13" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="F55" s="6" t="n">
-        <v>9000000</v>
+        <v>386500</v>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>Roger Gołombek</t>
+          <t>Agnieszka Zając</t>
         </is>
       </c>
     </row>
@@ -3194,12 +3198,12 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>2.5.2.3</t>
+          <t>5.13.2</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Supply of reinforcing steel</t>
+          <t>Auxiliary fuel tank (light oil/diesel oil)</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
@@ -3208,14 +3212,14 @@
         </is>
       </c>
       <c r="E56" s="13" t="n">
-        <v>46181</v>
+        <v>46189</v>
       </c>
       <c r="F56" s="6" t="n">
-        <v>386500</v>
+        <v>200000</v>
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>Agnieszka Zając</t>
+          <t>Magdalena Białorucka</t>
         </is>
       </c>
     </row>
@@ -3227,28 +3231,28 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>5.13.2</t>
+          <t>2.8.1</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Auxiliary fuel tank (light oil/diesel oil)</t>
+          <t>Parapet</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>enquiry</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="E57" s="13" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="F57" s="6" t="n">
-        <v>200000</v>
+        <v>82476</v>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>Magdalena Białorucka</t>
+          <t>Joanna Sawicka</t>
         </is>
       </c>
     </row>
@@ -3260,12 +3264,12 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>2.8.1</t>
+          <t>2.8.10</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Parapet</t>
+          <t>Soffit lining</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
@@ -3277,7 +3281,7 @@
         <v>46190</v>
       </c>
       <c r="F58" s="6" t="n">
-        <v>82476</v>
+        <v>308662.24</v>
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
@@ -3293,12 +3297,12 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>2.8.10</t>
+          <t>2.8.11</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Soffit lining</t>
+          <t>Scaffolding</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
@@ -3310,7 +3314,7 @@
         <v>46190</v>
       </c>
       <c r="F59" s="6" t="n">
-        <v>308662.24</v>
+        <v>77076</v>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
@@ -3326,12 +3330,12 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>2.8.11</t>
+          <t>2.8.12</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Scaffolding</t>
+          <t>Safety system</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
@@ -3343,7 +3347,7 @@
         <v>46190</v>
       </c>
       <c r="F60" s="6" t="n">
-        <v>77076</v>
+        <v>150018.35</v>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
@@ -3359,12 +3363,12 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>2.8.12</t>
+          <t>2.8.13</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Safety system</t>
+          <t>Shutters</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
@@ -3376,7 +3380,7 @@
         <v>46190</v>
       </c>
       <c r="F61" s="6" t="n">
-        <v>150018.35</v>
+        <v>107600.56</v>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
@@ -3392,12 +3396,12 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>2.8.13</t>
+          <t>2.8.2</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Shutters</t>
+          <t>Steel-aluminum canopy</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
@@ -3409,7 +3413,7 @@
         <v>46190</v>
       </c>
       <c r="F62" s="6" t="n">
-        <v>107600.56</v>
+        <v>120922.87</v>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
@@ -3425,12 +3429,12 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>2.8.2</t>
+          <t>2.8.3</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Steel-aluminum canopy</t>
+          <t>Aluminum-glass facade</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
@@ -3442,7 +3446,7 @@
         <v>46190</v>
       </c>
       <c r="F63" s="6" t="n">
-        <v>120922.87</v>
+        <v>296487.48</v>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
@@ -3458,12 +3462,12 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>2.8.3</t>
+          <t>2.8.4</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Aluminum-glass facade</t>
+          <t xml:space="preserve">ETICS </t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
@@ -3475,7 +3479,7 @@
         <v>46190</v>
       </c>
       <c r="F64" s="6" t="n">
-        <v>296487.48</v>
+        <v>122038.26</v>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
@@ -3491,12 +3495,12 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>2.8.4</t>
+          <t>2.8.5</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">ETICS </t>
+          <t>Flashings</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
@@ -3508,7 +3512,7 @@
         <v>46190</v>
       </c>
       <c r="F65" s="6" t="n">
-        <v>122038.26</v>
+        <v>366598.98</v>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
@@ -3524,12 +3528,12 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>2.8.5</t>
+          <t>2.8.6</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Flashings</t>
+          <t>Sheet metal cladding</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
@@ -3541,7 +3545,7 @@
         <v>46190</v>
       </c>
       <c r="F66" s="6" t="n">
-        <v>366598.98</v>
+        <v>1172886.87</v>
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
@@ -3557,24 +3561,24 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>2.8.6</t>
+          <t>2.8.7</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Sheet metal cladding</t>
+          <t>Sandwich panel cladding</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>enquiry</t>
         </is>
       </c>
       <c r="E67" s="13" t="n">
         <v>46190</v>
       </c>
       <c r="F67" s="6" t="n">
-        <v>1172886.87</v>
+        <v>5792279.88</v>
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
@@ -3590,24 +3594,24 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>2.8.7</t>
+          <t>2.8.8</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Sandwich panel cladding</t>
+          <t>Fiber cement panel cladding</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>enquiry</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="E68" s="13" t="n">
         <v>46190</v>
       </c>
       <c r="F68" s="6" t="n">
-        <v>5792279.88</v>
+        <v>241170.5</v>
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
@@ -3623,12 +3627,12 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>2.8.8</t>
+          <t>2.8.9</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Fiber cement panel cladding</t>
+          <t>Substructures</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
@@ -3640,7 +3644,7 @@
         <v>46190</v>
       </c>
       <c r="F69" s="6" t="n">
-        <v>241170.5</v>
+        <v>419580</v>
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
@@ -3656,12 +3660,12 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>2.8.9</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Substructures</t>
+          <t>Notification Bodies</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
@@ -3670,16 +3674,12 @@
         </is>
       </c>
       <c r="E70" s="13" t="n">
-        <v>46190</v>
+        <v>46201</v>
       </c>
       <c r="F70" s="6" t="n">
-        <v>419580</v>
-      </c>
-      <c r="G70" s="5" t="inlineStr">
-        <is>
-          <t>Joanna Sawicka</t>
-        </is>
-      </c>
+        <v>350000</v>
+      </c>
+      <c r="G70" s="5" t="n"/>
     </row>
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="5" t="inlineStr">
@@ -3689,24 +3689,24 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>2.5.1.4</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Notification Bodies</t>
+          <t>Execution of pre-wall insulation</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>negotiation</t>
         </is>
       </c>
       <c r="E71" s="13" t="n">
         <v>46201</v>
       </c>
       <c r="F71" s="6" t="n">
-        <v>350000</v>
+        <v>500000</v>
       </c>
       <c r="G71" s="5" t="n"/>
     </row>
@@ -3718,26 +3718,30 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>2.5.1.4</t>
+          <t>5.4.3</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Execution of pre-wall insulation</t>
+          <t>Fly ash extraction system for the boiler and conveyors</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>negotiation</t>
+          <t>enquiry</t>
         </is>
       </c>
       <c r="E72" s="13" t="n">
-        <v>46201</v>
+        <v>46202</v>
       </c>
       <c r="F72" s="6" t="n">
-        <v>500000</v>
-      </c>
-      <c r="G72" s="5" t="n"/>
+        <v>4260000</v>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>Roger Gołombek</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="20" customHeight="1">
       <c r="A73" s="5" t="inlineStr">
@@ -3747,30 +3751,26 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>5.4.3</t>
+          <t>1.2.6.2</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Fly ash extraction system for the boiler and conveyors</t>
+          <t>Piping design</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>enquiry</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="E73" s="13" t="n">
-        <v>46202</v>
+        <v>46205</v>
       </c>
       <c r="F73" s="6" t="n">
-        <v>4260000</v>
-      </c>
-      <c r="G73" s="5" t="inlineStr">
-        <is>
-          <t>Roger Gołombek</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G73" s="5" t="n"/>
     </row>
     <row r="74" ht="20" customHeight="1">
       <c r="A74" s="5" t="inlineStr">
@@ -3780,12 +3780,12 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>1.2.6.2</t>
+          <t>5.7.1</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Piping design</t>
+          <t>SNCR DeNOx system including silo, pumps</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
@@ -3797,9 +3797,13 @@
         <v>46205</v>
       </c>
       <c r="F74" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G74" s="5" t="n"/>
+        <v>1090000</v>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>Magdalena Białorucka</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="20" customHeight="1">
       <c r="A75" s="5" t="inlineStr">
@@ -3809,12 +3813,12 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>5.7.1</t>
+          <t>4.3.6</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>SNCR DeNOx system including silo, pumps</t>
+          <t>Emergency showers and eye washers</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
@@ -3823,14 +3827,14 @@
         </is>
       </c>
       <c r="E75" s="13" t="n">
-        <v>46205</v>
+        <v>46212</v>
       </c>
       <c r="F75" s="6" t="n">
-        <v>1090000</v>
+        <v>10000</v>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>Magdalena Białorucka</t>
+          <t>Magdalena Przeździak</t>
         </is>
       </c>
     </row>
@@ -3842,12 +3846,12 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>4.3.6</t>
+          <t>5.10.11</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Emergency showers and eye washers</t>
+          <t>Heat exchangers 2 pcs., LP pre-heater, external economizer</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
@@ -3856,14 +3860,14 @@
         </is>
       </c>
       <c r="E76" s="13" t="n">
-        <v>46212</v>
+        <v>46215</v>
       </c>
       <c r="F76" s="6" t="n">
-        <v>10000</v>
+        <v>3242866</v>
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>Magdalena Przeździak</t>
+          <t>Stanisław Rucki</t>
         </is>
       </c>
     </row>
@@ -3875,12 +3879,12 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>5.10.11</t>
+          <t>1.2.3</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Heat exchangers 2 pcs., LP pre-heater, external economizer</t>
+          <t>Detailed design: fire-fighting system</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
@@ -3889,16 +3893,12 @@
         </is>
       </c>
       <c r="E77" s="13" t="n">
-        <v>46215</v>
+        <v>46218</v>
       </c>
       <c r="F77" s="6" t="n">
-        <v>3242866</v>
-      </c>
-      <c r="G77" s="5" t="inlineStr">
-        <is>
-          <t>Stanisław Rucki</t>
-        </is>
-      </c>
+        <v>260000</v>
+      </c>
+      <c r="G77" s="5" t="n"/>
     </row>
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="5" t="inlineStr">
@@ -3908,12 +3908,12 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>1.2.3</t>
+          <t>4.3.1</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Detailed design: fire-fighting system</t>
+          <t>Boiler room roof ventilators and wall shutters</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
@@ -3925,9 +3925,13 @@
         <v>46218</v>
       </c>
       <c r="F78" s="6" t="n">
-        <v>260000</v>
-      </c>
-      <c r="G78" s="5" t="n"/>
+        <v>1500000</v>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>Magdalena Przeździak</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="5" t="inlineStr">
@@ -3937,12 +3941,12 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>4.3.1</t>
+          <t>4.3.2</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Boiler room roof ventilators and wall shutters</t>
+          <t>HVAC for the technological buildings</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
@@ -3954,7 +3958,7 @@
         <v>46218</v>
       </c>
       <c r="F79" s="6" t="n">
-        <v>1500000</v>
+        <v>3107033</v>
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
@@ -3970,12 +3974,12 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>4.3.2</t>
+          <t>4.3.3</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>HVAC for the technological buildings</t>
+          <t xml:space="preserve">HVAC for the other buildings </t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
@@ -3987,7 +3991,7 @@
         <v>46218</v>
       </c>
       <c r="F80" s="6" t="n">
-        <v>3107033</v>
+        <v>1548256</v>
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
@@ -4003,12 +4007,12 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>4.3.3</t>
+          <t>3.4.3</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">HVAC for the other buildings </t>
+          <t>Emission monitoring system (CEMS)</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
@@ -4017,14 +4021,14 @@
         </is>
       </c>
       <c r="E81" s="13" t="n">
-        <v>46218</v>
+        <v>46219</v>
       </c>
       <c r="F81" s="6" t="n">
-        <v>1548256</v>
+        <v>1960000</v>
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>Magdalena Przeździak</t>
+          <t>Radosław Zdancewicz</t>
         </is>
       </c>
     </row>
@@ -4036,28 +4040,28 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>3.4.3</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Emission monitoring system (CEMS)</t>
+          <t>Deodorization system</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>enquiry</t>
         </is>
       </c>
       <c r="E82" s="13" t="n">
         <v>46219</v>
       </c>
       <c r="F82" s="6" t="n">
-        <v>1960000</v>
+        <v>1009700</v>
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>Radosław Zdancewicz</t>
+          <t>Stanisław Rucki</t>
         </is>
       </c>
     </row>
@@ -4069,30 +4073,26 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>5.13.3</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Deodorization system</t>
+          <t>Light oil unloading installation with TDT documentation approval</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>enquiry</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="E83" s="13" t="n">
-        <v>46219</v>
+        <v>46222</v>
       </c>
       <c r="F83" s="6" t="n">
-        <v>1009700</v>
-      </c>
-      <c r="G83" s="5" t="inlineStr">
-        <is>
-          <t>Stanisław Rucki</t>
-        </is>
-      </c>
+        <v>200000</v>
+      </c>
+      <c r="G83" s="5" t="n"/>
     </row>
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="5" t="inlineStr">
@@ -4102,26 +4102,30 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>5.13.3</t>
+          <t>5.10.12</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Light oil unloading installation with TDT documentation approval</t>
+          <t>Stabilising pumps 2 x 100%, network pumps 3 x 50%, condensate pumps 2 x 100%, feed water pumps 3 pcs., cooling pumps</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>enquiry</t>
         </is>
       </c>
       <c r="E84" s="13" t="n">
-        <v>46222</v>
+        <v>46231</v>
       </c>
       <c r="F84" s="6" t="n">
-        <v>200000</v>
-      </c>
-      <c r="G84" s="5" t="n"/>
+        <v>5517325</v>
+      </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>Stanisław Rucki</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="20" customHeight="1">
       <c r="A85" s="5" t="inlineStr">
@@ -4131,24 +4135,24 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>5.10.12</t>
+          <t>5.13.4</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Stabilising pumps 2 x 100%, network pumps 3 x 50%, condensate pumps 2 x 100%, feed water pumps 3 pcs., cooling pumps</t>
+          <t>Auxiliary fuel pumps (light oil/diesel oil), demi water pumps, other water pumps</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>enquiry</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="E85" s="13" t="n">
         <v>46231</v>
       </c>
       <c r="F85" s="6" t="n">
-        <v>5517325</v>
+        <v>3337500</v>
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
@@ -4164,12 +4168,12 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>5.13.4</t>
+          <t>2.11.1</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Auxiliary fuel pumps (light oil/diesel oil), demi water pumps, other water pumps</t>
+          <t>Painting</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
@@ -4178,14 +4182,14 @@
         </is>
       </c>
       <c r="E86" s="13" t="n">
-        <v>46231</v>
+        <v>46234</v>
       </c>
       <c r="F86" s="6" t="n">
-        <v>3337500</v>
+        <v>669442.8</v>
       </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
-          <t>Stanisław Rucki</t>
+          <t>Magdalena Białorucka</t>
         </is>
       </c>
     </row>
@@ -4197,12 +4201,12 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>2.11.1</t>
+          <t>2.11.10</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Painting</t>
+          <t>Plasterboard wall, sandwich panel wall</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
@@ -4214,13 +4218,9 @@
         <v>46234</v>
       </c>
       <c r="F87" s="6" t="n">
-        <v>669442.8</v>
-      </c>
-      <c r="G87" s="5" t="inlineStr">
-        <is>
-          <t>Magdalena Białorucka</t>
-        </is>
-      </c>
+        <v>39026.75</v>
+      </c>
+      <c r="G87" s="5" t="n"/>
     </row>
     <row r="88" ht="20" customHeight="1">
       <c r="A88" s="5" t="inlineStr">
@@ -4230,12 +4230,12 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>2.11.10</t>
+          <t>2.11.11</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Plasterboard wall, sandwich panel wall</t>
+          <t>Glass wall</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
@@ -4247,7 +4247,7 @@
         <v>46234</v>
       </c>
       <c r="F88" s="6" t="n">
-        <v>39026.75</v>
+        <v>75045.3</v>
       </c>
       <c r="G88" s="5" t="n"/>
     </row>
@@ -4259,12 +4259,12 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>2.11.11</t>
+          <t>2.11.12</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Glass wall</t>
+          <t>Plastering</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
@@ -4276,9 +4276,13 @@
         <v>46234</v>
       </c>
       <c r="F89" s="6" t="n">
-        <v>75045.3</v>
-      </c>
-      <c r="G89" s="5" t="n"/>
+        <v>1241084.64</v>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>Magdalena Białorucka</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="20" customHeight="1">
       <c r="A90" s="5" t="inlineStr">
@@ -4288,12 +4292,12 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>2.11.12</t>
+          <t>2.11.13</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Plastering</t>
+          <t>Carpet / polyamide</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
@@ -4305,13 +4309,9 @@
         <v>46234</v>
       </c>
       <c r="F90" s="6" t="n">
-        <v>1241084.64</v>
-      </c>
-      <c r="G90" s="5" t="inlineStr">
-        <is>
-          <t>Magdalena Białorucka</t>
-        </is>
-      </c>
+        <v>87497.52</v>
+      </c>
+      <c r="G90" s="5" t="n"/>
     </row>
     <row r="91" ht="20" customHeight="1">
       <c r="A91" s="5" t="inlineStr">
@@ -4321,12 +4321,12 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>2.11.13</t>
+          <t>2.11.14</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Carpet / polyamide</t>
+          <t>Wall and column protection up to 2.5 m + hydrophobic protection</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
@@ -4338,7 +4338,7 @@
         <v>46234</v>
       </c>
       <c r="F91" s="6" t="n">
-        <v>87497.52</v>
+        <v>186490.48</v>
       </c>
       <c r="G91" s="5" t="n"/>
     </row>
@@ -4350,12 +4350,12 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>2.11.14</t>
+          <t>2.11.2</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>Wall and column protection up to 2.5 m + hydrophobic protection</t>
+          <t>Furniture</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
@@ -4367,9 +4367,13 @@
         <v>46234</v>
       </c>
       <c r="F92" s="6" t="n">
-        <v>186490.48</v>
-      </c>
-      <c r="G92" s="5" t="n"/>
+        <v>631074</v>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>Magdalena Białorucka</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="20" customHeight="1">
       <c r="A93" s="5" t="inlineStr">
@@ -4379,12 +4383,12 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>2.11.2</t>
+          <t>2.11.3</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Furniture</t>
+          <t>Tiles</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
@@ -4396,7 +4400,7 @@
         <v>46234</v>
       </c>
       <c r="F93" s="6" t="n">
-        <v>631074</v>
+        <v>498448.22</v>
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
@@ -4412,12 +4416,12 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>2.11.3</t>
+          <t>2.11.4</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>Tiles</t>
+          <t>Raised floor</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
@@ -4429,7 +4433,7 @@
         <v>46234</v>
       </c>
       <c r="F94" s="6" t="n">
-        <v>498448.22</v>
+        <v>621907.75</v>
       </c>
       <c r="G94" s="5" t="inlineStr">
         <is>
@@ -4445,30 +4449,26 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>2.11.4</t>
+          <t>2.11.5</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Raised floor</t>
+          <t>Concrete floor + screed</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>enquiry</t>
         </is>
       </c>
       <c r="E95" s="13" t="n">
         <v>46234</v>
       </c>
       <c r="F95" s="6" t="n">
-        <v>621907.75</v>
-      </c>
-      <c r="G95" s="5" t="inlineStr">
-        <is>
-          <t>Magdalena Białorucka</t>
-        </is>
-      </c>
+        <v>610629.23</v>
+      </c>
+      <c r="G95" s="5" t="n"/>
     </row>
     <row r="96" ht="20" customHeight="1">
       <c r="A96" s="5" t="inlineStr">
@@ -4478,24 +4478,24 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>2.11.5</t>
+          <t>2.11.5.4</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>Concrete floor + screed</t>
+          <t>Concrete flooring and screed with insulation</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>enquiry</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="E96" s="13" t="n">
         <v>46234</v>
       </c>
       <c r="F96" s="6" t="n">
-        <v>610629.23</v>
+        <v>0</v>
       </c>
       <c r="G96" s="5" t="n"/>
     </row>
@@ -4507,12 +4507,12 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>2.11.5.4</t>
+          <t>2.11.6</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Concrete flooring and screed with insulation</t>
+          <t>Microcement floor</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
@@ -4524,7 +4524,7 @@
         <v>46234</v>
       </c>
       <c r="F97" s="6" t="n">
-        <v>0</v>
+        <v>133705.44</v>
       </c>
       <c r="G97" s="5" t="n"/>
     </row>
@@ -4536,12 +4536,12 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>2.11.6</t>
+          <t>2.11.7</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>Microcement floor</t>
+          <t>Resin floor</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
@@ -4553,9 +4553,13 @@
         <v>46234</v>
       </c>
       <c r="F98" s="6" t="n">
-        <v>133705.44</v>
-      </c>
-      <c r="G98" s="5" t="n"/>
+        <v>655174.75</v>
+      </c>
+      <c r="G98" s="5" t="inlineStr">
+        <is>
+          <t>Magdalena Białorucka</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="20" customHeight="1">
       <c r="A99" s="5" t="inlineStr">
@@ -4565,12 +4569,12 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>2.11.7</t>
+          <t>2.11.8</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Resin floor</t>
+          <t>Suspended ceilings</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
@@ -4582,13 +4586,9 @@
         <v>46234</v>
       </c>
       <c r="F99" s="6" t="n">
-        <v>655174.75</v>
-      </c>
-      <c r="G99" s="5" t="inlineStr">
-        <is>
-          <t>Magdalena Białorucka</t>
-        </is>
-      </c>
+        <v>220670.05</v>
+      </c>
+      <c r="G99" s="5" t="n"/>
     </row>
     <row r="100" ht="20" customHeight="1">
       <c r="A100" s="5" t="inlineStr">
@@ -4598,12 +4598,12 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>2.11.8</t>
+          <t>2.11.9</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>Suspended ceilings</t>
+          <t>Segmented sliding wall</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
@@ -4615,7 +4615,7 @@
         <v>46234</v>
       </c>
       <c r="F100" s="6" t="n">
-        <v>220670.05</v>
+        <v>65014.1</v>
       </c>
       <c r="G100" s="5" t="n"/>
     </row>
@@ -4627,26 +4627,30 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>2.11.9</t>
+          <t>2.12.1</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Segmented sliding wall</t>
+          <t>Passenger and good elevator</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>enquiry</t>
         </is>
       </c>
       <c r="E101" s="13" t="n">
         <v>46234</v>
       </c>
       <c r="F101" s="6" t="n">
-        <v>65014.1</v>
-      </c>
-      <c r="G101" s="5" t="n"/>
+        <v>415350</v>
+      </c>
+      <c r="G101" s="5" t="inlineStr">
+        <is>
+          <t>Izabela Malarecka</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="20" customHeight="1">
       <c r="A102" s="5" t="inlineStr">
@@ -4656,12 +4660,12 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>2.12.1</t>
+          <t>2.12.2</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>Passenger and good elevator</t>
+          <t>Passenger elevator</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
@@ -4673,7 +4677,7 @@
         <v>46234</v>
       </c>
       <c r="F102" s="6" t="n">
-        <v>415350</v>
+        <v>98643.60000000001</v>
       </c>
       <c r="G102" s="5" t="inlineStr">
         <is>
@@ -4689,28 +4693,28 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>2.12.2</t>
+          <t>2.13</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Passenger elevator</t>
+          <t>Weigh bridge</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>enquiry</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="E103" s="13" t="n">
         <v>46234</v>
       </c>
       <c r="F103" s="6" t="n">
-        <v>98643.60000000001</v>
+        <v>551900</v>
       </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
-          <t>Izabela Malarecka</t>
+          <t>Stanisław Rucki</t>
         </is>
       </c>
     </row>
@@ -4722,12 +4726,12 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>2.13</t>
+          <t>5.14.2</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>Weigh bridge</t>
+          <t>Mechanical installation of technological equipment</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
@@ -4739,7 +4743,7 @@
         <v>46234</v>
       </c>
       <c r="F104" s="6" t="n">
-        <v>551900</v>
+        <v>1500000</v>
       </c>
       <c r="G104" s="5" t="inlineStr">
         <is>
@@ -4755,12 +4759,12 @@
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>5.14.2</t>
+          <t>5.4.6</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Mechanical installation of technological equipment</t>
+          <t>Compensator between boiler and ECO</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
@@ -4772,13 +4776,9 @@
         <v>46234</v>
       </c>
       <c r="F105" s="6" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="G105" s="5" t="inlineStr">
-        <is>
-          <t>Stanisław Rucki</t>
-        </is>
-      </c>
+        <v>129000</v>
+      </c>
+      <c r="G105" s="5" t="n"/>
     </row>
     <row r="106" ht="20" customHeight="1">
       <c r="A106" s="5" t="inlineStr">
@@ -4788,12 +4788,12 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>5.4.6</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>Compensator between boiler and ECO</t>
+          <t>Refractory</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
@@ -4805,9 +4805,13 @@
         <v>46234</v>
       </c>
       <c r="F106" s="6" t="n">
-        <v>129000</v>
-      </c>
-      <c r="G106" s="5" t="n"/>
+        <v>3993000</v>
+      </c>
+      <c r="G106" s="5" t="inlineStr">
+        <is>
+          <t>Magdalena Białorucka</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="20" customHeight="1">
       <c r="A107" s="5" t="inlineStr">
@@ -4817,24 +4821,24 @@
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>4.2.2</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Refractory</t>
+          <t>Firefighting water tank</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>enquiry</t>
         </is>
       </c>
       <c r="E107" s="13" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="F107" s="6" t="n">
-        <v>3993000</v>
+        <v>275700</v>
       </c>
       <c r="G107" s="5" t="inlineStr">
         <is>
@@ -4850,28 +4854,28 @@
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>4.2.2</t>
+          <t>5.13.1</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>Firefighting water tank</t>
+          <t>Compressors 2 x 50% + 1 x 50%</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>enquiry</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="E108" s="13" t="n">
         <v>46235</v>
       </c>
       <c r="F108" s="6" t="n">
-        <v>275700</v>
+        <v>1500000</v>
       </c>
       <c r="G108" s="5" t="inlineStr">
         <is>
-          <t>Magdalena Białorucka</t>
+          <t>Roger Gołombek</t>
         </is>
       </c>
     </row>
@@ -4883,12 +4887,12 @@
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>5.13.1</t>
+          <t>4.3.5</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Compressors 2 x 50% + 1 x 50%</t>
+          <t>Sanitary water, connection to source, storage, pumping, underground and external distribution</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
@@ -4897,14 +4901,14 @@
         </is>
       </c>
       <c r="E109" s="13" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="F109" s="6" t="n">
-        <v>1500000</v>
+        <v>637613</v>
       </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
-          <t>Roger Gołombek</t>
+          <t>Magdalena Przeździak</t>
         </is>
       </c>
     </row>
@@ -4916,12 +4920,12 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>4.3.5</t>
+          <t>4.3.7</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>Sanitary water, connection to source, storage, pumping, underground and external distribution</t>
+          <t>Sanitary waste water collection, treatment and connection to discharge point</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
@@ -4933,7 +4937,7 @@
         <v>46236</v>
       </c>
       <c r="F110" s="6" t="n">
-        <v>637613</v>
+        <v>624272</v>
       </c>
       <c r="G110" s="5" t="inlineStr">
         <is>
@@ -4949,12 +4953,12 @@
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>4.3.7</t>
+          <t>4.3.8</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Sanitary waste water collection, treatment and connection to discharge point</t>
+          <t>Waste water collection and connection to discharge point</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
@@ -4966,7 +4970,7 @@
         <v>46236</v>
       </c>
       <c r="F111" s="6" t="n">
-        <v>624272</v>
+        <v>200969</v>
       </c>
       <c r="G111" s="5" t="inlineStr">
         <is>
@@ -4982,12 +4986,12 @@
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>4.3.8</t>
+          <t>4.3.9</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
-          <t>Waste water collection and connection to discharge point</t>
+          <t>Rain water and snowmelt collection, treatment and connection to discharge point</t>
         </is>
       </c>
       <c r="D112" s="5" t="inlineStr">
@@ -4999,7 +5003,7 @@
         <v>46236</v>
       </c>
       <c r="F112" s="6" t="n">
-        <v>200969</v>
+        <v>3359643</v>
       </c>
       <c r="G112" s="5" t="inlineStr">
         <is>
@@ -5015,12 +5019,12 @@
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>4.3.9</t>
+          <t>5.13.9</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Rain water and snowmelt collection, treatment and connection to discharge point</t>
+          <t>Grate cooling system</t>
         </is>
       </c>
       <c r="D113" s="5" t="inlineStr">
@@ -5032,11 +5036,11 @@
         <v>46236</v>
       </c>
       <c r="F113" s="6" t="n">
-        <v>3359643</v>
+        <v>731000</v>
       </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
-          <t>Magdalena Przeździak</t>
+          <t>Magdalena Białorucka</t>
         </is>
       </c>
     </row>
@@ -5048,12 +5052,12 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>5.13.9</t>
+          <t>2.6.4</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>Grate cooling system</t>
+          <t>Steel structure of the staircase in the B1.4 facility (change from the reinforced concrete structure in relation to the acquisition stage)</t>
         </is>
       </c>
       <c r="D114" s="5" t="inlineStr">
@@ -5062,14 +5066,14 @@
         </is>
       </c>
       <c r="E114" s="13" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="F114" s="6" t="n">
-        <v>731000</v>
+        <v>470146.23</v>
       </c>
       <c r="G114" s="5" t="inlineStr">
         <is>
-          <t>Magdalena Białorucka</t>
+          <t>Robert Klimczak</t>
         </is>
       </c>
     </row>
@@ -5081,12 +5085,12 @@
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>2.6.4</t>
+          <t>3.4.2</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Steel structure of the staircase in the B1.4 facility (change from the reinforced concrete structure in relation to the acquisition stage)</t>
+          <t>DCS System</t>
         </is>
       </c>
       <c r="D115" s="5" t="inlineStr">
@@ -5095,14 +5099,14 @@
         </is>
       </c>
       <c r="E115" s="13" t="n">
-        <v>46237</v>
+        <v>46250</v>
       </c>
       <c r="F115" s="6" t="n">
-        <v>470146.23</v>
+        <v>2752000</v>
       </c>
       <c r="G115" s="5" t="inlineStr">
         <is>
-          <t>Robert Klimczak</t>
+          <t>Roger Gołombek</t>
         </is>
       </c>
     </row>
@@ -5114,12 +5118,12 @@
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>3.4.2</t>
+          <t>5.7.4</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>DCS System</t>
+          <t>Fly ash silos</t>
         </is>
       </c>
       <c r="D116" s="5" t="inlineStr">
@@ -5131,7 +5135,7 @@
         <v>46250</v>
       </c>
       <c r="F116" s="6" t="n">
-        <v>2752000</v>
+        <v>2000000</v>
       </c>
       <c r="G116" s="5" t="inlineStr">
         <is>
@@ -5147,12 +5151,12 @@
       </c>
       <c r="B117" s="5" t="inlineStr">
         <is>
-          <t>5.7.4</t>
+          <t>5.10.7</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Fly ash silos</t>
+          <t>Main cooler</t>
         </is>
       </c>
       <c r="D117" s="5" t="inlineStr">
@@ -5161,7 +5165,7 @@
         </is>
       </c>
       <c r="E117" s="13" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="F117" s="6" t="n">
         <v>2000000</v>
@@ -5180,12 +5184,12 @@
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>5.10.7</t>
+          <t>5.10.8</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>Main cooler</t>
+          <t>Cooler tank, condensate tank</t>
         </is>
       </c>
       <c r="D118" s="5" t="inlineStr">
@@ -5197,7 +5201,7 @@
         <v>46251</v>
       </c>
       <c r="F118" s="6" t="n">
-        <v>2000000</v>
+        <v>1000000</v>
       </c>
       <c r="G118" s="5" t="inlineStr">
         <is>
@@ -5213,12 +5217,12 @@
       </c>
       <c r="B119" s="5" t="inlineStr">
         <is>
-          <t>5.10.8</t>
+          <t>5.13.11</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Cooler tank, condensate tank</t>
+          <t>waste water treatment</t>
         </is>
       </c>
       <c r="D119" s="5" t="inlineStr">
@@ -5230,7 +5234,7 @@
         <v>46251</v>
       </c>
       <c r="F119" s="6" t="n">
-        <v>1000000</v>
+        <v>800000</v>
       </c>
       <c r="G119" s="5" t="inlineStr">
         <is>
@@ -5246,12 +5250,12 @@
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>5.13.11</t>
+          <t>5.4.5</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>waste water treatment</t>
+          <t>Chemical dosing for the boiler</t>
         </is>
       </c>
       <c r="D120" s="5" t="inlineStr">
@@ -5263,11 +5267,11 @@
         <v>46251</v>
       </c>
       <c r="F120" s="6" t="n">
-        <v>800000</v>
+        <v>223600</v>
       </c>
       <c r="G120" s="5" t="inlineStr">
         <is>
-          <t>Roger Gołombek</t>
+          <t>Magdalena Białorucka</t>
         </is>
       </c>
     </row>
@@ -5279,59 +5283,26 @@
       </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
-          <t>5.4.5</t>
+          <t>5.10.9</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Chemical dosing for the boiler</t>
+          <t>Water pressure stabilization system</t>
         </is>
       </c>
       <c r="D121" s="5" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>negotiation</t>
         </is>
       </c>
       <c r="E121" s="13" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="F121" s="6" t="n">
-        <v>223600</v>
-      </c>
-      <c r="G121" s="5" t="inlineStr">
-        <is>
-          <t>Magdalena Białorucka</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="20" customHeight="1">
-      <c r="A122" s="5" t="inlineStr">
-        <is>
-          <t>Next orders 3 months</t>
-        </is>
-      </c>
-      <c r="B122" s="5" t="inlineStr">
-        <is>
-          <t>5.10.9</t>
-        </is>
-      </c>
-      <c r="C122" s="5" t="inlineStr">
-        <is>
-          <t>Water pressure stabilization system</t>
-        </is>
-      </c>
-      <c r="D122" s="5" t="inlineStr">
-        <is>
-          <t>negotiation</t>
-        </is>
-      </c>
-      <c r="E122" s="13" t="n">
-        <v>46252</v>
-      </c>
-      <c r="F122" s="6" t="n">
         <v>350000</v>
       </c>
-      <c r="G122" s="5" t="n"/>
+      <c r="G121" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8503,7 +8474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G122"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -12149,36 +12120,6 @@
       </c>
       <c r="G121" s="5">
         <f>'10_Source_Orders_3M'!G121</f>
-        <v/>
-      </c>
-    </row>
-    <row r="122" ht="20" customHeight="1">
-      <c r="A122" s="5">
-        <f>'10_Source_Orders_3M'!A122</f>
-        <v/>
-      </c>
-      <c r="B122" s="5">
-        <f>'10_Source_Orders_3M'!B122</f>
-        <v/>
-      </c>
-      <c r="C122" s="5">
-        <f>'10_Source_Orders_3M'!C122</f>
-        <v/>
-      </c>
-      <c r="D122" s="5">
-        <f>'10_Source_Orders_3M'!D122</f>
-        <v/>
-      </c>
-      <c r="E122" s="13">
-        <f>'10_Source_Orders_3M'!E122</f>
-        <v/>
-      </c>
-      <c r="F122" s="6">
-        <f>'10_Source_Orders_3M'!F122</f>
-        <v/>
-      </c>
-      <c r="G122" s="5">
-        <f>'10_Source_Orders_3M'!G122</f>
         <v/>
       </c>
     </row>

</xml_diff>